<commit_message>
refactor: rename placa to señal
</commit_message>
<xml_diff>
--- a/Plan Prod mayo 2026.xlsx
+++ b/Plan Prod mayo 2026.xlsx
@@ -475,7 +475,7 @@
     <t>Carenaje</t>
   </si>
   <si>
-    <t>Placas</t>
+    <t>Señales</t>
   </si>
   <si>
     <t>Tubos</t>
@@ -520,7 +520,7 @@
     <t>Banco olímpico inclinado</t>
   </si>
   <si>
-    <t>Banco predicador con placas</t>
+    <t>Banco predicador con señales</t>
   </si>
   <si>
     <t xml:space="preserve">fondos triceps peso libre </t>
@@ -784,7 +784,7 @@
     <t>XM193</t>
   </si>
   <si>
-    <t>Hammer isolateral vuelos con placas</t>
+    <t>Hammer isolateral vuelos con señales</t>
   </si>
   <si>
     <t>Arrastrar</t>
@@ -1087,7 +1087,7 @@
     <t>XB429</t>
   </si>
   <si>
-    <t>Placa Informativa Individual</t>
+    <t>Señal Informativa Individual</t>
   </si>
   <si>
     <t>XB430</t>

</xml_diff>